<commit_message>
Leite assignedGroups bei Touren und Kursen aus der Kategorie ab
Mit der Sektion Trier abgesprochen: Die Gruppe ergibt sich aus der Kategorie
(mapping.yaml, kategorie.*.gruppe) und ersetzt die Formularspalte 'Gruppen'.
Kategorien ohne feste Gruppe (z.B. Ski) bleiben leer.
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/kurse_tr.xlsx
+++ b/tests/fixtures/expected/kurse_tr.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>/264 - Sektion Trier/Gruppen/Klettern</t>
+          <t>/264 - Sektion Trier/Gruppen/Bergsteigen</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -904,7 +904,11 @@
           <t>&lt;p&gt;&amp;nbsp;&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>/264 - Sektion Trier/Gruppen/Wandergruppe</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t>/264 - Sektion Trier/Personen/Personen/Max Mustermann</t>

</xml_diff>

<commit_message>
Gib Termine ohne Ende nur mit Start aus, Ende mit 00:00:00
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/kurse_tr.xlsx
+++ b/tests/fixtures/expected/kurse_tr.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 23:59:59</t>
+          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 00:00:00</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 23:59:59</t>
+          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 00:00:00</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 23:59:59</t>
+          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 00:00:00</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 23:59:59</t>
+          <t>[dates]2026-10-10 00:00:00 bis 2026-10-11 00:00:00</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">

</xml_diff>